<commit_message>
Refine quote flow and profile layout
</commit_message>
<xml_diff>
--- a/profiles/koncept/quotation-layout.xlsx
+++ b/profiles/koncept/quotation-layout.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>ESTIMATE</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Attention:</t>
   </si>
   <si>
-    <t xml:space="preserve">RE: </t>
+    <t xml:space="preserve"/>
   </si>
   <si>
     <t>Pos.</t>
@@ -49,21 +49,12 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Terms &amp; Conditions :</t>
-  </si>
-  <si>
     <t>80% payment upon confirmation and signing of contract.</t>
   </si>
   <si>
     <t>20% balance 7 days after delivery.</t>
   </si>
   <si>
-    <t>All cheques should be crossed and made payable to Koncept Image Pte Ltd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note : </t>
-  </si>
-  <si>
     <t>The above contract does not include application fees to any relevant authorities and electrical connection fees.</t>
   </si>
   <si>
@@ -73,9 +64,6 @@
     <t>Any changes agreed upon after the confirmation of contract or during the work in progress shall be deemed as Additional Orders.</t>
   </si>
   <si>
-    <t>We accept the quotation amount and the terms</t>
-  </si>
-  <si>
     <t>All designs and dimensions are subject to final site verification.</t>
   </si>
   <si>
@@ -94,9 +82,6 @@
     <t>All deposit are non-refundable upon of cancellation of agreement.</t>
   </si>
   <si>
-    <t>The client is obliged to adhere to the above payment terms &amp; conditions of  works.</t>
-  </si>
-  <si>
     <t>11.00</t>
   </si>
   <si>
@@ -106,25 +91,10 @@
     <t>Late payment charge of 1.5% per month will be charge after the due date.</t>
   </si>
   <si>
-    <t>Koncept Image Pte Ltd</t>
-  </si>
-  <si>
     <t>_____________________________</t>
   </si>
   <si>
     <t>_____________________________________</t>
-  </si>
-  <si>
-    <t>Francies Cheng</t>
-  </si>
-  <si>
-    <t>Person in charge</t>
-  </si>
-  <si>
-    <t>Company name &amp; stamp</t>
-  </si>
-  <si>
-    <t>Date:</t>
   </si>
 </sst>
 </file>
@@ -622,7 +592,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:ns2="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
@@ -641,7 +611,7 @@
         <xdr:cNvPr id="3" name="Rectangle 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <ns2:creationId id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -676,7 +646,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Koncept Image Pte Limited</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -692,7 +662,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>61 Kaki Bukit Ave 1, #02-26,</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -708,7 +678,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Shunli Industrial Park</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -724,7 +694,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Singapore 417943</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -740,7 +710,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Telephone: +6568177477</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -772,7 +742,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Bank Detail:</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -789,7 +759,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>United Overseas Bank Limited</a:t>
+            <a:t/>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="900" b="0" i="0" baseline="0">
@@ -797,7 +767,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>, </a:t>
+            <a:t/>
           </a:r>
           <a:r>
             <a:rPr lang="en-SG" sz="900" b="0" i="0">
@@ -806,7 +776,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>80 Raffles Place</a:t>
+            <a:t/>
           </a:r>
         </a:p>
         <a:p>
@@ -818,7 +788,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Singapore 048624</a:t>
+            <a:t/>
           </a:r>
         </a:p>
         <a:p>
@@ -829,7 +799,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Account: 335-3020-445</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -845,7 +815,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Swift Code: UOVBSGSG</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US" sz="900">
             <a:latin typeface="+mn-lt"/>
@@ -876,7 +846,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Project No: </a:t>
+            <a:t/>
           </a:r>
         </a:p>
         <a:p>
@@ -899,7 +869,7 @@
             <a:rPr lang="en-SG" sz="800">
               <a:latin typeface="Chaparral Pro" pitchFamily="18" charset="0"/>
             </a:rPr>
-            <a:t> </a:t>
+            <a:t/>
           </a:r>
         </a:p>
         <a:p>
@@ -914,58 +884,6 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1676400</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>200025</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6833" name="Picture 7" descr="KonceptWorld logo.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-0000B11A0000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="6686550" y="323850"/>
-          <a:ext cx="1647825" cy="352425"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1318,13 +1236,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U146"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="17" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.125" style="8" customWidth="1"/>
     <col min="2" max="2" width="10.5" style="13" customWidth="1"/>
@@ -1345,7 +1263,7 @@
     <col min="18" max="16384" width="9.125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
@@ -1357,7 +1275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
@@ -1367,7 +1285,7 @@
       <c r="H2" s="7"/>
       <c r="I2" s="8"/>
     </row>
-    <row r="3" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
@@ -1377,7 +1295,7 @@
       <c r="H3" s="7"/>
       <c r="I3" s="8"/>
     </row>
-    <row r="4" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
@@ -1387,7 +1305,7 @@
       <c r="H4" s="7"/>
       <c r="I4" s="8"/>
     </row>
-    <row r="5" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.25">
       <c r="B5" s="35"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -1397,7 +1315,7 @@
       <c r="H5" s="7"/>
       <c r="I5" s="8"/>
     </row>
-    <row r="6" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A6" s="12"/>
       <c r="B6" s="5"/>
       <c r="E6" s="5"/>
@@ -1406,7 +1324,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A7" s="90"/>
       <c r="B7" s="5"/>
       <c r="E7" s="5"/>
@@ -1415,7 +1333,7 @@
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A8" s="89"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -1423,7 +1341,7 @@
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A9" s="67"/>
       <c r="B9" s="5"/>
       <c r="E9" s="5"/>
@@ -1432,7 +1350,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
     </row>
-    <row r="10" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A10" s="69"/>
       <c r="B10" s="36"/>
       <c r="C10" s="10"/>
@@ -1443,7 +1361,7 @@
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
     </row>
-    <row r="11" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A11" s="67"/>
       <c r="B11" s="22"/>
       <c r="C11" s="18"/>
@@ -1452,7 +1370,7 @@
       <c r="G11" s="6"/>
       <c r="I11" s="8"/>
     </row>
-    <row r="12" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A12" s="26" t="s">
         <v>1</v>
       </c>
@@ -1463,7 +1381,7 @@
       <c r="G12" s="6"/>
       <c r="I12" s="8"/>
     </row>
-    <row r="13" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A13" s="23"/>
       <c r="B13" s="24"/>
       <c r="C13" s="21"/>
@@ -1472,7 +1390,7 @@
       <c r="G13" s="6"/>
       <c r="I13" s="8"/>
     </row>
-    <row r="14" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A14" s="23"/>
       <c r="B14" s="24"/>
       <c r="C14" s="21"/>
@@ -1481,7 +1399,7 @@
       <c r="G14" s="6"/>
       <c r="I14" s="8"/>
     </row>
-    <row r="15" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A15" s="25"/>
       <c r="B15" s="24"/>
       <c r="C15" s="21"/>
@@ -1490,7 +1408,7 @@
       <c r="G15" s="6"/>
       <c r="I15" s="8"/>
     </row>
-    <row r="16" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A16" s="98">
         <v>46176</v>
       </c>
@@ -1501,7 +1419,7 @@
       <c r="G16" s="6"/>
       <c r="I16" s="8"/>
     </row>
-    <row r="17" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A17" s="23"/>
       <c r="B17" s="24"/>
       <c r="C17" s="21"/>
@@ -1510,7 +1428,7 @@
       <c r="G17" s="6"/>
       <c r="I17" s="8"/>
     </row>
-    <row r="18" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A18" s="26" t="s">
         <v>2</v>
       </c>
@@ -1521,7 +1439,7 @@
       <c r="G18" s="6"/>
       <c r="I18" s="8"/>
     </row>
-    <row r="19" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A19" s="23"/>
       <c r="B19" s="24"/>
       <c r="C19" s="21"/>
@@ -1530,7 +1448,7 @@
       <c r="G19" s="6"/>
       <c r="I19" s="8"/>
     </row>
-    <row r="20" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A20" s="23" t="s">
         <v>3</v>
       </c>
@@ -1547,7 +1465,7 @@
       <c r="G20" s="6"/>
       <c r="I20" s="6"/>
     </row>
-    <row r="21" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A21" s="27"/>
       <c r="B21" s="24"/>
       <c r="C21" s="21"/>
@@ -1556,35 +1474,35 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A22" s="28"/>
       <c r="B22" s="18"/>
       <c r="C22" s="81"/>
       <c r="D22" s="21"/>
       <c r="E22" s="22"/>
     </row>
-    <row r="23" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A23" s="27"/>
       <c r="B23" s="24"/>
       <c r="C23" s="21"/>
       <c r="D23" s="21"/>
       <c r="E23" s="22"/>
     </row>
-    <row r="24" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A24" s="27"/>
       <c r="B24" s="70"/>
       <c r="C24" s="24"/>
       <c r="D24" s="21"/>
       <c r="E24" s="22"/>
     </row>
-    <row r="25" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A25" s="27"/>
       <c r="B25" s="24"/>
       <c r="C25" s="24"/>
       <c r="D25" s="21"/>
       <c r="E25" s="22"/>
     </row>
-    <row r="26" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A26" s="27"/>
       <c r="B26" s="70"/>
       <c r="C26" s="21"/>
@@ -1592,7 +1510,7 @@
       <c r="E26" s="22"/>
       <c r="L26" s="71"/>
     </row>
-    <row r="27" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A27" s="27"/>
       <c r="B27" s="24"/>
       <c r="C27" s="21"/>
@@ -1600,7 +1518,7 @@
       <c r="E27" s="22"/>
       <c r="L27" s="71"/>
     </row>
-    <row r="28" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A28" s="28"/>
       <c r="B28" s="29"/>
       <c r="C28" s="18"/>
@@ -1608,102 +1526,102 @@
       <c r="E28" s="30"/>
       <c r="F28" s="91"/>
     </row>
-    <row r="29" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A29" s="28"/>
       <c r="B29" s="29"/>
       <c r="C29" s="18"/>
       <c r="D29" s="24"/>
       <c r="E29" s="30"/>
     </row>
-    <row r="30" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A30" s="27"/>
       <c r="D30" s="24"/>
       <c r="E30" s="30"/>
     </row>
-    <row r="31" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A31" s="28"/>
       <c r="D31" s="24"/>
       <c r="E31" s="30"/>
     </row>
-    <row r="32" spans="1:12" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A32" s="28"/>
       <c r="D32" s="24"/>
       <c r="E32" s="30"/>
     </row>
-    <row r="33" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A33" s="28"/>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
     </row>
-    <row r="34" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D34" s="34"/>
       <c r="G34" s="5"/>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
     </row>
-    <row r="35" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D35" s="34"/>
       <c r="G35" s="5"/>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
     </row>
-    <row r="36" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D36" s="34"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
     </row>
-    <row r="37" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D37" s="34"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
       <c r="I37" s="5"/>
     </row>
-    <row r="38" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D38" s="34"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
     </row>
-    <row r="39" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D39" s="34"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
     </row>
-    <row r="40" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D40" s="34"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
     </row>
-    <row r="41" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D41" s="34"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
     </row>
-    <row r="42" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D42" s="34"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
     </row>
-    <row r="43" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D43" s="34"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5"/>
       <c r="I43" s="5"/>
     </row>
-    <row r="44" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D44" s="34"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5"/>
       <c r="I44" s="5"/>
     </row>
-    <row r="45" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A45" s="80"/>
       <c r="B45" s="7"/>
       <c r="C45" s="12"/>
@@ -1712,50 +1630,50 @@
       <c r="H45" s="5"/>
       <c r="I45" s="5"/>
     </row>
-    <row r="46" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="B46" s="7"/>
       <c r="D46" s="34"/>
       <c r="G46" s="5"/>
       <c r="H46" s="5"/>
       <c r="I46" s="5"/>
     </row>
-    <row r="47" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D47" s="34"/>
       <c r="G47" s="5"/>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
     </row>
-    <row r="48" spans="1:9" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D48" s="34"/>
       <c r="G48" s="5"/>
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
     </row>
-    <row r="49" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D49" s="34"/>
       <c r="G49" s="5"/>
       <c r="H49" s="5"/>
       <c r="I49" s="5"/>
     </row>
-    <row r="50" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D50" s="34"/>
       <c r="G50" s="5"/>
       <c r="H50" s="5"/>
       <c r="I50" s="5"/>
     </row>
-    <row r="51" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D51" s="34"/>
       <c r="G51" s="5"/>
       <c r="H51" s="5"/>
       <c r="I51" s="5"/>
     </row>
-    <row r="52" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D52" s="34"/>
       <c r="G52" s="5"/>
       <c r="H52" s="5"/>
       <c r="I52" s="5"/>
     </row>
-    <row r="53" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A53" s="23" t="s">
         <v>3</v>
       </c>
@@ -1772,7 +1690,7 @@
       <c r="G53" s="6"/>
       <c r="I53" s="6"/>
     </row>
-    <row r="54" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A54" s="23"/>
       <c r="B54" s="24"/>
       <c r="C54" s="21"/>
@@ -1781,7 +1699,7 @@
       <c r="G54" s="6"/>
       <c r="I54" s="6"/>
     </row>
-    <row r="55" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A55" s="28"/>
       <c r="B55" s="5"/>
       <c r="C55" s="18"/>
@@ -1789,38 +1707,38 @@
       <c r="G55" s="6"/>
       <c r="I55" s="6"/>
     </row>
-    <row r="56" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A56" s="5"/>
       <c r="B56" s="5"/>
       <c r="E56" s="5"/>
       <c r="G56" s="6"/>
       <c r="I56" s="6"/>
     </row>
-    <row r="57" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A57" s="68"/>
       <c r="E57" s="93"/>
       <c r="G57" s="6"/>
       <c r="I57" s="6"/>
     </row>
-    <row r="58" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A58" s="68"/>
       <c r="E58" s="5"/>
       <c r="G58" s="6"/>
       <c r="I58" s="6"/>
     </row>
-    <row r="59" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A59" s="68"/>
       <c r="E59" s="94"/>
       <c r="G59" s="6"/>
       <c r="I59" s="6"/>
     </row>
-    <row r="60" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.3">
       <c r="A60" s="68"/>
       <c r="E60" s="5"/>
       <c r="G60" s="6"/>
       <c r="I60" s="6"/>
     </row>
-    <row r="61" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A61" s="28"/>
       <c r="B61" s="5"/>
       <c r="C61" s="18"/>
@@ -1830,42 +1748,42 @@
       <c r="I61" s="5"/>
       <c r="J61" s="5"/>
     </row>
-    <row r="62" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
       <c r="H62" s="5"/>
       <c r="I62" s="5"/>
       <c r="J62" s="5"/>
     </row>
-    <row r="63" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="E63" s="84"/>
       <c r="F63" s="5"/>
       <c r="G63" s="5"/>
       <c r="H63" s="5"/>
       <c r="I63" s="5"/>
     </row>
-    <row r="64" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="E64" s="84"/>
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" s="5"/>
       <c r="I64" s="5"/>
     </row>
-    <row r="65" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D65" s="34"/>
       <c r="E65" s="84"/>
       <c r="Q65" s="8"/>
       <c r="R65" s="13"/>
       <c r="U65" s="15"/>
     </row>
-    <row r="66" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D66" s="34"/>
       <c r="E66" s="84"/>
       <c r="Q66" s="8"/>
       <c r="R66" s="13"/>
       <c r="U66" s="15"/>
     </row>
-    <row r="67" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A67" s="87"/>
       <c r="D67" s="34"/>
       <c r="E67" s="84"/>
@@ -1873,7 +1791,7 @@
       <c r="R67" s="13"/>
       <c r="U67" s="15"/>
     </row>
-    <row r="68" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A68" s="86"/>
       <c r="D68" s="34"/>
       <c r="E68" s="84"/>
@@ -1881,7 +1799,7 @@
       <c r="R68" s="13"/>
       <c r="U68" s="15"/>
     </row>
-    <row r="69" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A69" s="83"/>
       <c r="C69" s="12"/>
       <c r="D69" s="34"/>
@@ -1891,7 +1809,7 @@
       <c r="R69" s="13"/>
       <c r="U69" s="15"/>
     </row>
-    <row r="70" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D70" s="34"/>
       <c r="E70" s="84"/>
       <c r="J70" s="5"/>
@@ -1899,49 +1817,49 @@
       <c r="R70" s="13"/>
       <c r="U70" s="15"/>
     </row>
-    <row r="71" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D71" s="34"/>
       <c r="E71" s="84"/>
       <c r="Q71" s="8"/>
       <c r="R71" s="13"/>
       <c r="U71" s="15"/>
     </row>
-    <row r="72" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D72" s="34"/>
       <c r="E72" s="84"/>
       <c r="Q72" s="8"/>
       <c r="R72" s="13"/>
       <c r="U72" s="15"/>
     </row>
-    <row r="73" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D73" s="34"/>
       <c r="E73" s="84"/>
       <c r="Q73" s="8"/>
       <c r="R73" s="13"/>
       <c r="U73" s="15"/>
     </row>
-    <row r="74" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D74" s="34"/>
       <c r="E74" s="84"/>
       <c r="Q74" s="8"/>
       <c r="R74" s="13"/>
       <c r="U74" s="15"/>
     </row>
-    <row r="75" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D75" s="34"/>
       <c r="E75" s="84"/>
       <c r="Q75" s="8"/>
       <c r="R75" s="13"/>
       <c r="U75" s="15"/>
     </row>
-    <row r="76" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D76" s="34"/>
       <c r="E76" s="84"/>
       <c r="Q76" s="8"/>
       <c r="R76" s="13"/>
       <c r="U76" s="15"/>
     </row>
-    <row r="77" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A77" s="28"/>
       <c r="B77" s="5"/>
       <c r="C77" s="18"/>
@@ -1951,7 +1869,7 @@
       <c r="H77" s="5"/>
       <c r="I77" s="5"/>
     </row>
-    <row r="78" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A78" s="28"/>
       <c r="B78" s="5"/>
       <c r="C78" s="96"/>
@@ -1961,7 +1879,7 @@
       <c r="H78" s="5"/>
       <c r="I78" s="5"/>
     </row>
-    <row r="79" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A79" s="5"/>
       <c r="B79" s="5"/>
       <c r="D79" s="7"/>
@@ -1971,7 +1889,7 @@
       <c r="H79" s="5"/>
       <c r="I79" s="5"/>
     </row>
-    <row r="80" spans="1:21" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:21" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D80" s="7"/>
       <c r="E80" s="95"/>
       <c r="F80" s="5"/>
@@ -1979,7 +1897,7 @@
       <c r="H80" s="5"/>
       <c r="I80" s="5"/>
     </row>
-    <row r="81" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D81" s="7"/>
       <c r="E81" s="31"/>
       <c r="F81" s="5"/>
@@ -1987,7 +1905,7 @@
       <c r="H81" s="5"/>
       <c r="I81" s="5"/>
     </row>
-    <row r="82" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D82" s="7"/>
       <c r="E82" s="95"/>
       <c r="F82" s="5"/>
@@ -1995,7 +1913,7 @@
       <c r="H82" s="5"/>
       <c r="I82" s="5"/>
     </row>
-    <row r="83" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="B83" s="5"/>
       <c r="D83" s="7"/>
       <c r="E83" s="31"/>
@@ -2004,7 +1922,7 @@
       <c r="H83" s="5"/>
       <c r="I83" s="5"/>
     </row>
-    <row r="84" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D84" s="7"/>
       <c r="E84" s="95"/>
       <c r="F84" s="5"/>
@@ -2012,7 +1930,7 @@
       <c r="H84" s="5"/>
       <c r="I84" s="5"/>
     </row>
-    <row r="85" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="D85" s="7"/>
       <c r="E85" s="31"/>
       <c r="F85" s="5"/>
@@ -2020,7 +1938,7 @@
       <c r="H85" s="5"/>
       <c r="I85" s="5"/>
     </row>
-    <row r="86" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A86" s="28"/>
       <c r="C86" s="18"/>
       <c r="E86" s="13"/>
@@ -2029,36 +1947,36 @@
       <c r="H86" s="5"/>
       <c r="I86" s="5"/>
     </row>
-    <row r="87" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="A87" s="5"/>
       <c r="D87" s="7"/>
       <c r="E87" s="31"/>
     </row>
-    <row r="88" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="E88" s="5"/>
     </row>
-    <row r="89" spans="1:10" ht="18.7" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" ht="18.7" customHeight="1" ns3:dyDescent="0.2">
       <c r="B89" s="5"/>
       <c r="E89" s="5"/>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:10" ns3:dyDescent="0.2">
       <c r="A90" s="28"/>
       <c r="C90" s="18"/>
       <c r="E90" s="5"/>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10" ns3:dyDescent="0.2">
       <c r="A91" s="5"/>
       <c r="D91" s="7"/>
       <c r="E91" s="31"/>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:10" ns3:dyDescent="0.2">
       <c r="D92" s="15"/>
       <c r="E92" s="94"/>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" ns3:dyDescent="0.2">
       <c r="C93" s="88"/>
     </row>
-    <row r="94" spans="1:10" ht="17.7" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" ht="17.7" thickBot="1" ns3:dyDescent="0.25">
       <c r="D94" s="34" t="s">
         <v>8</v>
       </c>
@@ -2071,34 +1989,31 @@
       </c>
       <c r="J94" s="79"/>
     </row>
-    <row r="95" spans="1:10" ht="17.7" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" ht="17.7" thickTop="1" ns3:dyDescent="0.2">
       <c r="B95" s="82"/>
       <c r="C95" s="12"/>
       <c r="D95" s="34"/>
       <c r="J95" s="79"/>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10" ns3:dyDescent="0.2">
       <c r="B96" s="82"/>
       <c r="C96" s="12"/>
       <c r="D96" s="34"/>
       <c r="J96" s="79"/>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:10" ns3:dyDescent="0.2">
       <c r="B97" s="82"/>
       <c r="C97" s="97"/>
       <c r="D97" s="34"/>
       <c r="J97" s="79"/>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10" ns3:dyDescent="0.2">
       <c r="B98" s="82"/>
       <c r="C98" s="12"/>
       <c r="D98" s="34"/>
       <c r="J98" s="79"/>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A99" s="37" t="s">
-        <v>9</v>
-      </c>
+    <row r="99" spans="1:10" ns3:dyDescent="0.2">
       <c r="B99" s="32"/>
       <c r="C99" s="41"/>
       <c r="D99" s="53"/>
@@ -2108,12 +2023,12 @@
       <c r="H99" s="38"/>
       <c r="I99" s="39"/>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:10" ns3:dyDescent="0.2">
       <c r="A100" s="40">
         <v>1</v>
       </c>
       <c r="B100" s="41" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C100" s="52"/>
       <c r="D100" s="42"/>
@@ -2123,12 +2038,12 @@
       <c r="H100" s="43"/>
       <c r="I100" s="45"/>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10" ns3:dyDescent="0.2">
       <c r="A101" s="40">
         <v>2</v>
       </c>
       <c r="B101" s="41" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C101" s="41"/>
       <c r="D101" s="42"/>
@@ -2138,11 +2053,8 @@
       <c r="H101" s="43"/>
       <c r="I101" s="45"/>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" ns3:dyDescent="0.25">
       <c r="A102" s="40"/>
-      <c r="B102" s="41" t="s">
-        <v>12</v>
-      </c>
       <c r="C102" s="41"/>
       <c r="D102" s="58"/>
       <c r="E102" s="2"/>
@@ -2151,10 +2063,7 @@
       <c r="H102" s="17"/>
       <c r="I102" s="17"/>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A103" s="46" t="s">
-        <v>13</v>
-      </c>
+    <row r="103" spans="1:10" ns3:dyDescent="0.2">
       <c r="B103" s="41"/>
       <c r="C103" s="2"/>
       <c r="D103" s="58"/>
@@ -2164,12 +2073,12 @@
       <c r="H103" s="48"/>
       <c r="I103" s="49"/>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" ns3:dyDescent="0.25">
       <c r="A104" s="40">
         <v>1</v>
       </c>
       <c r="B104" s="41" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" s="62"/>
@@ -2179,12 +2088,12 @@
       <c r="H104" s="48"/>
       <c r="I104" s="49"/>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" ns3:dyDescent="0.25">
       <c r="A105" s="40">
         <v>2</v>
       </c>
       <c r="B105" s="41" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C105" s="17"/>
       <c r="D105" s="58"/>
@@ -2194,29 +2103,26 @@
       <c r="H105" s="50"/>
       <c r="I105" s="16"/>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:10" ns3:dyDescent="0.2">
       <c r="A106" s="40">
         <v>3</v>
       </c>
       <c r="B106" s="41" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" s="65"/>
-      <c r="E106" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="F106" s="51"/>
       <c r="G106" s="50"/>
       <c r="H106" s="50"/>
       <c r="I106" s="16"/>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:10" ns3:dyDescent="0.2">
       <c r="A107" s="40">
         <v>4</v>
       </c>
       <c r="B107" s="41" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" s="2"/>
@@ -2226,12 +2132,12 @@
       <c r="H107" s="48"/>
       <c r="I107" s="49"/>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:10" ns3:dyDescent="0.2">
       <c r="A108" s="40">
         <v>5</v>
       </c>
       <c r="B108" s="41" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" s="2"/>
@@ -2241,12 +2147,12 @@
       <c r="H108" s="56"/>
       <c r="I108" s="57"/>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:10" ns3:dyDescent="0.2">
       <c r="A109" s="40">
         <v>6</v>
       </c>
       <c r="B109" s="41" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" s="2"/>
@@ -2256,12 +2162,12 @@
       <c r="H109" s="48"/>
       <c r="I109" s="49"/>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10" ns3:dyDescent="0.2">
       <c r="A110" s="40">
         <v>7</v>
       </c>
       <c r="B110" s="41" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" s="2"/>
@@ -2271,42 +2177,39 @@
       <c r="H110" s="1"/>
       <c r="I110" s="1"/>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:10" ns3:dyDescent="0.2">
       <c r="A111" s="40">
         <v>8</v>
       </c>
       <c r="B111" s="41" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" s="2"/>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:10" ns3:dyDescent="0.2">
       <c r="A112" s="40">
         <v>9</v>
       </c>
       <c r="B112" s="41" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:10" ns3:dyDescent="0.2">
       <c r="A113" s="40">
         <v>10</v>
       </c>
-      <c r="B113" s="41" t="s">
-        <v>24</v>
-      </c>
       <c r="C113" s="2"/>
       <c r="D113" s="2"/>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:10" ns3:dyDescent="0.2">
       <c r="A114" s="46" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B114" s="41" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C114" s="2"/>
       <c r="F114" s="64"/>
@@ -2314,10 +2217,10 @@
       <c r="H114" s="3"/>
       <c r="I114" s="2"/>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:10" ns3:dyDescent="0.2">
       <c r="A115" s="33"/>
       <c r="B115" s="41" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C115" s="2"/>
       <c r="F115" s="64"/>
@@ -2325,7 +2228,7 @@
       <c r="H115" s="3"/>
       <c r="I115" s="2"/>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:10" ns3:dyDescent="0.2">
       <c r="A116" s="33"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
@@ -2334,37 +2237,34 @@
       <c r="H116" s="3"/>
       <c r="I116" s="2"/>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:10" ns3:dyDescent="0.2">
       <c r="A117" s="33"/>
-      <c r="B117" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="F117" s="59"/>
       <c r="G117" s="60"/>
       <c r="H117" s="61"/>
       <c r="I117" s="2"/>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:10" ns3:dyDescent="0.2">
       <c r="A118" s="33"/>
       <c r="B118" s="61"/>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:10" ns3:dyDescent="0.2">
       <c r="A119" s="33"/>
       <c r="B119" s="61"/>
       <c r="J119" s="72"/>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:10" ns3:dyDescent="0.2">
       <c r="A120" s="33"/>
       <c r="B120" s="61"/>
       <c r="J120" s="73"/>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:10" ns3:dyDescent="0.2">
       <c r="A121" s="33"/>
       <c r="B121" s="33" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E121" s="65" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F121" s="43"/>
       <c r="G121" s="47"/>
@@ -2372,103 +2272,91 @@
       <c r="I121" s="49"/>
       <c r="J121" s="73"/>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" ns3:dyDescent="0.25">
       <c r="A122" s="33"/>
-      <c r="B122" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="E122" s="65" t="s">
-        <v>32</v>
-      </c>
       <c r="F122" s="59"/>
       <c r="G122" s="60"/>
       <c r="H122" s="61"/>
       <c r="I122" s="2"/>
       <c r="J122" s="74"/>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:10" ns3:dyDescent="0.2">
       <c r="B123" s="61"/>
-      <c r="E123" s="65" t="s">
-        <v>33</v>
-      </c>
       <c r="F123" s="59"/>
       <c r="G123" s="60"/>
       <c r="H123" s="61"/>
       <c r="I123" s="2"/>
       <c r="J123" s="75"/>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" ns3:dyDescent="0.25">
       <c r="B124" s="61"/>
-      <c r="E124" s="65" t="s">
-        <v>34</v>
-      </c>
       <c r="F124" s="63"/>
       <c r="G124" s="17"/>
       <c r="H124" s="17"/>
       <c r="I124" s="17"/>
       <c r="J124" s="75"/>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:10" ns3:dyDescent="0.2">
       <c r="F125" s="5"/>
       <c r="G125" s="5"/>
       <c r="H125" s="5"/>
       <c r="J125" s="76"/>
     </row>
-    <row r="126" spans="1:10" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:10" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J126" s="76"/>
     </row>
-    <row r="127" spans="1:10" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:10" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J127" s="75"/>
     </row>
-    <row r="128" spans="1:10" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:10" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J128" s="77"/>
     </row>
-    <row r="129" spans="6:11" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="6:11" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J129" s="75"/>
     </row>
-    <row r="130" spans="6:11" s="1" customFormat="1" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="6:11" s="1" customFormat="1" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J130" s="75"/>
       <c r="K130" s="77"/>
     </row>
-    <row r="131" spans="6:11" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="6:11" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J131" s="78"/>
     </row>
-    <row r="132" spans="6:11" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="6:11" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J132" s="78"/>
     </row>
-    <row r="133" spans="6:11" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="6:11" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.25">
       <c r="J133" s="74"/>
     </row>
-    <row r="134" spans="6:11" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="6:11" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J134" s="78"/>
     </row>
-    <row r="135" spans="6:11" ht="17.350000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="6:11" ht="17.350000000000001" customHeight="1" ns3:dyDescent="0.2">
       <c r="J135" s="78"/>
     </row>
-    <row r="136" spans="6:11" x14ac:dyDescent="0.2">
+    <row r="136" spans="6:11" ns3:dyDescent="0.2">
       <c r="J136" s="78"/>
     </row>
-    <row r="137" spans="6:11" x14ac:dyDescent="0.2">
+    <row r="137" spans="6:11" ns3:dyDescent="0.2">
       <c r="J137" s="78"/>
     </row>
-    <row r="138" spans="6:11" x14ac:dyDescent="0.2">
+    <row r="138" spans="6:11" ns3:dyDescent="0.2">
       <c r="J138" s="78"/>
     </row>
-    <row r="139" spans="6:11" x14ac:dyDescent="0.2">
+    <row r="139" spans="6:11" ns3:dyDescent="0.2">
       <c r="J139" s="78"/>
     </row>
-    <row r="140" spans="6:11" x14ac:dyDescent="0.2">
+    <row r="140" spans="6:11" ns3:dyDescent="0.2">
       <c r="J140" s="78"/>
     </row>
-    <row r="144" spans="6:11" x14ac:dyDescent="0.2">
+    <row r="144" spans="6:11" ns3:dyDescent="0.2">
       <c r="F144" s="5"/>
       <c r="G144" s="5"/>
       <c r="H144" s="5"/>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" ns3:dyDescent="0.2">
       <c r="A145" s="13"/>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" ns3:dyDescent="0.2">
       <c r="F146" s="5"/>
     </row>
   </sheetData>

</xml_diff>